<commit_message>
Ajustes robustos no processamento de NF-e, cálculo de custo fracionado e automação da alimentação de produtos_processados. Auditoria e melhoria de lógica centralizadas.
</commit_message>
<xml_diff>
--- a/Custos Anúncios Shopee.xlsx
+++ b/Custos Anúncios Shopee.xlsx
@@ -25,7 +25,7 @@
     <t>CÓD. REFERÊNCIA VARIAÇÃO</t>
   </si>
   <si>
-    <t>CUSTO</t>
+    <t>Custo Real (NF)</t>
   </si>
   <si>
     <t>ANG0217</t>
@@ -2691,7 +2691,7 @@
     <col customWidth="1" min="2" max="2" width="18.0"/>
     <col customWidth="1" min="3" max="3" width="21.56"/>
     <col customWidth="1" min="4" max="4" width="22.11"/>
-    <col customWidth="1" min="5" max="5" width="7.11"/>
+    <col customWidth="1" min="5" max="5" width="12.11"/>
     <col customWidth="1" min="6" max="6" width="11.22"/>
   </cols>
   <sheetData>
@@ -2724,19 +2724,19 @@
       <c r="Z1" s="1"/>
     </row>
     <row r="2">
-      <c r="A2" s="1" t="s">
+      <c r="A2" s="3" t="s">
         <v>0</v>
       </c>
-      <c r="B2" s="1" t="s">
+      <c r="B2" s="3" t="s">
         <v>1</v>
       </c>
-      <c r="C2" s="1" t="s">
+      <c r="C2" s="3" t="s">
         <v>2</v>
       </c>
-      <c r="D2" s="2" t="s">
+      <c r="D2" s="4" t="s">
         <v>3</v>
       </c>
-      <c r="E2" s="1" t="s">
+      <c r="E2" s="3" t="s">
         <v>4</v>
       </c>
       <c r="F2" s="1"/>
@@ -2965,7 +2965,7 @@
         <v>10</v>
       </c>
       <c r="E8" s="3">
-        <v>88.96</v>
+        <v>90.37</v>
       </c>
       <c r="F8" s="1"/>
       <c r="G8" s="1"/>
@@ -3117,7 +3117,7 @@
         <v>14</v>
       </c>
       <c r="E12" s="3">
-        <v>9.2</v>
+        <v>9.1</v>
       </c>
       <c r="F12" s="1"/>
       <c r="G12" s="1"/>
@@ -3231,7 +3231,7 @@
         <v>17</v>
       </c>
       <c r="E15" s="3">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="F15" s="1"/>
       <c r="G15" s="1"/>
@@ -5359,7 +5359,7 @@
         <v>72</v>
       </c>
       <c r="E71" s="3">
-        <v>38.2</v>
+        <v>33.09</v>
       </c>
       <c r="F71" s="1"/>
       <c r="G71" s="1"/>
@@ -5625,7 +5625,7 @@
         <v>79</v>
       </c>
       <c r="E78" s="3">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="F78" s="1"/>
       <c r="G78" s="1"/>
@@ -5739,7 +5739,7 @@
         <v>83</v>
       </c>
       <c r="E81" s="3">
-        <v>4.5</v>
+        <v>4.4</v>
       </c>
       <c r="F81" s="1"/>
       <c r="G81" s="1"/>
@@ -5815,7 +5815,7 @@
         <v>86</v>
       </c>
       <c r="E83" s="3">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="F83" s="1"/>
       <c r="G83" s="1"/>
@@ -6537,7 +6537,7 @@
         <v>104</v>
       </c>
       <c r="E102" s="3">
-        <v>12.5</v>
+        <v>12.3</v>
       </c>
       <c r="F102" s="1"/>
       <c r="G102" s="1"/>
@@ -6575,7 +6575,7 @@
         <v>105</v>
       </c>
       <c r="E103" s="3">
-        <v>21.35</v>
+        <v>20.45</v>
       </c>
       <c r="F103" s="1"/>
       <c r="G103" s="1"/>
@@ -6613,7 +6613,7 @@
         <v>107</v>
       </c>
       <c r="E104" s="3">
-        <v>13.6</v>
+        <v>13.2</v>
       </c>
       <c r="F104" s="1"/>
       <c r="G104" s="1"/>
@@ -6689,7 +6689,7 @@
         <v>109</v>
       </c>
       <c r="E106" s="3">
-        <v>23.0</v>
+        <v>22.8</v>
       </c>
       <c r="F106" s="1"/>
       <c r="G106" s="1"/>
@@ -6727,7 +6727,7 @@
         <v>110</v>
       </c>
       <c r="E107" s="3">
-        <v>42.42</v>
+        <v>45.6</v>
       </c>
       <c r="F107" s="1"/>
       <c r="G107" s="1"/>
@@ -6765,7 +6765,7 @@
         <v>110</v>
       </c>
       <c r="E108" s="3">
-        <v>42.42</v>
+        <v>45.6</v>
       </c>
       <c r="F108" s="1"/>
       <c r="G108" s="1"/>
@@ -6841,7 +6841,7 @@
         <v>114</v>
       </c>
       <c r="E110" s="3">
-        <v>26.2</v>
+        <v>26.0</v>
       </c>
       <c r="F110" s="1"/>
       <c r="G110" s="1"/>
@@ -7031,7 +7031,7 @@
         <v>119</v>
       </c>
       <c r="E115" s="3">
-        <v>27.8</v>
+        <v>27.6</v>
       </c>
       <c r="F115" s="1"/>
       <c r="G115" s="1"/>
@@ -7069,7 +7069,7 @@
         <v>119</v>
       </c>
       <c r="E116" s="3">
-        <v>27.8</v>
+        <v>27.6</v>
       </c>
       <c r="F116" s="1"/>
       <c r="G116" s="1"/>
@@ -7145,7 +7145,7 @@
         <v>113</v>
       </c>
       <c r="E118" s="3">
-        <v>39.3</v>
+        <v>39.0</v>
       </c>
       <c r="F118" s="1"/>
       <c r="G118" s="1"/>
@@ -7183,7 +7183,7 @@
         <v>121</v>
       </c>
       <c r="E119" s="3">
-        <v>63.62</v>
+        <v>68.4</v>
       </c>
       <c r="F119" s="1"/>
       <c r="G119" s="1"/>
@@ -7221,7 +7221,7 @@
         <v>121</v>
       </c>
       <c r="E120" s="3">
-        <v>63.62</v>
+        <v>68.4</v>
       </c>
       <c r="F120" s="1"/>
       <c r="G120" s="1"/>
@@ -7601,7 +7601,7 @@
         <v>130</v>
       </c>
       <c r="E130" s="3">
-        <v>9.0</v>
+        <v>8.8</v>
       </c>
       <c r="F130" s="1"/>
       <c r="G130" s="1"/>
@@ -7867,7 +7867,7 @@
         <v>135</v>
       </c>
       <c r="E137" s="3">
-        <v>25.0</v>
+        <v>24.6</v>
       </c>
       <c r="F137" s="1"/>
       <c r="G137" s="1"/>
@@ -7905,7 +7905,7 @@
         <v>136</v>
       </c>
       <c r="E138" s="3">
-        <v>40.5</v>
+        <v>40.2</v>
       </c>
       <c r="F138" s="1"/>
       <c r="G138" s="1"/>
@@ -7943,7 +7943,7 @@
         <v>136</v>
       </c>
       <c r="E139" s="3">
-        <v>40.5</v>
+        <v>40.2</v>
       </c>
       <c r="F139" s="1"/>
       <c r="G139" s="1"/>
@@ -8209,7 +8209,7 @@
         <v>143</v>
       </c>
       <c r="E146" s="3">
-        <v>18.9</v>
+        <v>17.67</v>
       </c>
       <c r="F146" s="1"/>
       <c r="G146" s="1"/>
@@ -8285,7 +8285,7 @@
         <v>145</v>
       </c>
       <c r="E148" s="3">
-        <v>13.5</v>
+        <v>13.2</v>
       </c>
       <c r="F148" s="1"/>
       <c r="G148" s="1"/>
@@ -8551,7 +8551,7 @@
         <v>149</v>
       </c>
       <c r="E155" s="3">
-        <v>37.5</v>
+        <v>36.9</v>
       </c>
       <c r="F155" s="1"/>
       <c r="G155" s="1"/>
@@ -8589,7 +8589,7 @@
         <v>150</v>
       </c>
       <c r="E156" s="3">
-        <v>11.6</v>
+        <v>11.1</v>
       </c>
       <c r="F156" s="1"/>
       <c r="G156" s="1"/>
@@ -8703,7 +8703,7 @@
         <v>153</v>
       </c>
       <c r="E159" s="3">
-        <v>18.0</v>
+        <v>17.6</v>
       </c>
       <c r="F159" s="1"/>
       <c r="G159" s="1"/>
@@ -8855,7 +8855,7 @@
         <v>157</v>
       </c>
       <c r="E163" s="3">
-        <v>10.5</v>
+        <v>9.9</v>
       </c>
       <c r="F163" s="1"/>
       <c r="G163" s="1"/>
@@ -9045,7 +9045,7 @@
         <v>82</v>
       </c>
       <c r="E168" s="3">
-        <v>22.5</v>
+        <v>22.0</v>
       </c>
       <c r="F168" s="1"/>
       <c r="G168" s="1"/>
@@ -9083,7 +9083,7 @@
         <v>106</v>
       </c>
       <c r="E169" s="3">
-        <v>6.8</v>
+        <v>6.6</v>
       </c>
       <c r="F169" s="1"/>
       <c r="G169" s="1"/>
@@ -9121,7 +9121,7 @@
         <v>161</v>
       </c>
       <c r="E170" s="3">
-        <v>13.4</v>
+        <v>12.9</v>
       </c>
       <c r="F170" s="1"/>
       <c r="G170" s="1"/>
@@ -9159,7 +9159,7 @@
         <v>162</v>
       </c>
       <c r="E171" s="3">
-        <v>11.5</v>
+        <v>11.4</v>
       </c>
       <c r="F171" s="1"/>
       <c r="G171" s="1"/>
@@ -9197,7 +9197,7 @@
         <v>111</v>
       </c>
       <c r="E172" s="3">
-        <v>21.21</v>
+        <v>22.8</v>
       </c>
       <c r="F172" s="1"/>
       <c r="G172" s="1"/>
@@ -9235,7 +9235,7 @@
         <v>111</v>
       </c>
       <c r="E173" s="3">
-        <v>21.21</v>
+        <v>22.8</v>
       </c>
       <c r="F173" s="1"/>
       <c r="G173" s="1"/>
@@ -9311,7 +9311,7 @@
         <v>164</v>
       </c>
       <c r="E175" s="3">
-        <v>13.1</v>
+        <v>13.0</v>
       </c>
       <c r="F175" s="1"/>
       <c r="G175" s="1"/>
@@ -9349,7 +9349,7 @@
         <v>165</v>
       </c>
       <c r="E176" s="3">
-        <v>13.8</v>
+        <v>13.7</v>
       </c>
       <c r="F176" s="1"/>
       <c r="G176" s="1"/>
@@ -9501,7 +9501,7 @@
         <v>118</v>
       </c>
       <c r="E180" s="3">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="F180" s="1"/>
       <c r="G180" s="1"/>
@@ -9539,7 +9539,7 @@
         <v>118</v>
       </c>
       <c r="E181" s="3">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="F181" s="1"/>
       <c r="G181" s="1"/>
@@ -9691,7 +9691,7 @@
         <v>172</v>
       </c>
       <c r="E185" s="3">
-        <v>68.12</v>
+        <v>69.6</v>
       </c>
       <c r="F185" s="1"/>
       <c r="G185" s="1"/>
@@ -9729,7 +9729,7 @@
         <v>173</v>
       </c>
       <c r="E186" s="3">
-        <v>34.06</v>
+        <v>34.8</v>
       </c>
       <c r="F186" s="1"/>
       <c r="G186" s="1"/>
@@ -9767,7 +9767,7 @@
         <v>174</v>
       </c>
       <c r="E187" s="3">
-        <v>21.0</v>
+        <v>19.8</v>
       </c>
       <c r="F187" s="1"/>
       <c r="G187" s="1"/>
@@ -9805,7 +9805,7 @@
         <v>174</v>
       </c>
       <c r="E188" s="3">
-        <v>21.0</v>
+        <v>19.8</v>
       </c>
       <c r="F188" s="1"/>
       <c r="G188" s="1"/>
@@ -9881,7 +9881,7 @@
         <v>176</v>
       </c>
       <c r="E190" s="3">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="F190" s="1"/>
       <c r="G190" s="1"/>
@@ -9995,7 +9995,7 @@
         <v>179</v>
       </c>
       <c r="E193" s="3">
-        <v>19.3</v>
+        <v>18.8</v>
       </c>
       <c r="F193" s="1"/>
       <c r="G193" s="1"/>
@@ -10033,7 +10033,7 @@
         <v>180</v>
       </c>
       <c r="E194" s="3">
-        <v>36.8</v>
+        <v>31.82</v>
       </c>
       <c r="F194" s="1"/>
       <c r="G194" s="1"/>
@@ -10071,7 +10071,7 @@
         <v>181</v>
       </c>
       <c r="E195" s="3">
-        <v>31.5</v>
+        <v>29.7</v>
       </c>
       <c r="F195" s="1"/>
       <c r="G195" s="1"/>
@@ -10109,7 +10109,7 @@
         <v>182</v>
       </c>
       <c r="E196" s="3">
-        <v>55.36</v>
+        <v>47.59</v>
       </c>
       <c r="F196" s="1"/>
       <c r="G196" s="1"/>
@@ -10223,7 +10223,7 @@
         <v>185</v>
       </c>
       <c r="E199" s="3">
-        <v>37.58</v>
+        <v>37.19</v>
       </c>
       <c r="F199" s="1"/>
       <c r="G199" s="1"/>
@@ -10337,7 +10337,7 @@
         <v>188</v>
       </c>
       <c r="E202" s="3">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="F202" s="1"/>
       <c r="G202" s="1"/>
@@ -10793,7 +10793,7 @@
         <v>200</v>
       </c>
       <c r="E214" s="3">
-        <v>21.45</v>
+        <v>21.3</v>
       </c>
       <c r="F214" s="1"/>
       <c r="G214" s="1"/>
@@ -10831,7 +10831,7 @@
         <v>201</v>
       </c>
       <c r="E215" s="3">
-        <v>21.95</v>
+        <v>21.55</v>
       </c>
       <c r="F215" s="1"/>
       <c r="G215" s="1"/>
@@ -10869,7 +10869,7 @@
         <v>202</v>
       </c>
       <c r="E216" s="3">
-        <v>29.65</v>
+        <v>28.5</v>
       </c>
       <c r="F216" s="1"/>
       <c r="G216" s="1"/>
@@ -10907,7 +10907,7 @@
         <v>203</v>
       </c>
       <c r="E217" s="3">
-        <v>28.58</v>
+        <v>28.19</v>
       </c>
       <c r="F217" s="1"/>
       <c r="G217" s="1"/>
@@ -10945,7 +10945,7 @@
         <v>204</v>
       </c>
       <c r="E218" s="3">
-        <v>25.6</v>
+        <v>25.35</v>
       </c>
       <c r="F218" s="1"/>
       <c r="G218" s="1"/>
@@ -10983,7 +10983,7 @@
         <v>205</v>
       </c>
       <c r="E219" s="3">
-        <v>26.68</v>
+        <v>26.29</v>
       </c>
       <c r="F219" s="1"/>
       <c r="G219" s="1"/>
@@ -11021,7 +11021,7 @@
         <v>206</v>
       </c>
       <c r="E220" s="3">
-        <v>24.31</v>
+        <v>23.9</v>
       </c>
       <c r="F220" s="1"/>
       <c r="G220" s="1"/>
@@ -11211,7 +11211,7 @@
         <v>211</v>
       </c>
       <c r="E225" s="3">
-        <v>14.1</v>
+        <v>14.0</v>
       </c>
       <c r="F225" s="1"/>
       <c r="G225" s="1"/>
@@ -11248,9 +11248,7 @@
       <c r="D226" s="4" t="s">
         <v>212</v>
       </c>
-      <c r="E226" s="3">
-        <v>13.0</v>
-      </c>
+      <c r="E226" s="3"/>
       <c r="F226" s="1"/>
       <c r="G226" s="1"/>
       <c r="H226" s="1"/>
@@ -11287,7 +11285,7 @@
         <v>213</v>
       </c>
       <c r="E227" s="3">
-        <v>27.27</v>
+        <v>26.86</v>
       </c>
       <c r="F227" s="1"/>
       <c r="G227" s="1"/>
@@ -11363,7 +11361,7 @@
         <v>214</v>
       </c>
       <c r="E229" s="3">
-        <v>27.2</v>
+        <v>27.0</v>
       </c>
       <c r="F229" s="1"/>
       <c r="G229" s="1"/>
@@ -12159,7 +12157,7 @@
         <v>233</v>
       </c>
       <c r="E250" s="3">
-        <v>13.5</v>
+        <v>12.5</v>
       </c>
       <c r="F250" s="1"/>
       <c r="G250" s="1"/>
@@ -14324,9 +14322,7 @@
       <c r="D307" s="4" t="s">
         <v>276</v>
       </c>
-      <c r="E307" s="3">
-        <v>13.0</v>
-      </c>
+      <c r="E307" s="3"/>
       <c r="F307" s="1"/>
       <c r="G307" s="1"/>
       <c r="H307" s="1"/>
@@ -16833,7 +16829,7 @@
         <v>314</v>
       </c>
       <c r="E373" s="3">
-        <v>31.14</v>
+        <v>31.04</v>
       </c>
       <c r="F373" s="1"/>
       <c r="G373" s="1"/>
@@ -16871,7 +16867,7 @@
         <v>315</v>
       </c>
       <c r="E374" s="3">
-        <v>31.1</v>
+        <v>30.1</v>
       </c>
       <c r="F374" s="1"/>
       <c r="G374" s="1"/>
@@ -16909,7 +16905,7 @@
         <v>79</v>
       </c>
       <c r="E375" s="3">
-        <v>18.8</v>
+        <v>18.6</v>
       </c>
       <c r="F375" s="1"/>
       <c r="G375" s="1"/>
@@ -16947,7 +16943,7 @@
         <v>316</v>
       </c>
       <c r="E376" s="3">
-        <v>16.67</v>
+        <v>16.46</v>
       </c>
       <c r="F376" s="1"/>
       <c r="G376" s="1"/>
@@ -17213,7 +17209,7 @@
         <v>322</v>
       </c>
       <c r="E383" s="3">
-        <v>29.84</v>
+        <v>30.64</v>
       </c>
       <c r="F383" s="1"/>
       <c r="G383" s="1"/>
@@ -17251,7 +17247,7 @@
         <v>110</v>
       </c>
       <c r="E384" s="3">
-        <v>42.42</v>
+        <v>45.6</v>
       </c>
       <c r="F384" s="1"/>
       <c r="G384" s="1"/>
@@ -17289,7 +17285,7 @@
         <v>119</v>
       </c>
       <c r="E385" s="3">
-        <v>27.8</v>
+        <v>27.6</v>
       </c>
       <c r="F385" s="1"/>
       <c r="G385" s="1"/>
@@ -17327,7 +17323,7 @@
         <v>121</v>
       </c>
       <c r="E386" s="3">
-        <v>63.62</v>
+        <v>68.4</v>
       </c>
       <c r="F386" s="1"/>
       <c r="G386" s="1"/>
@@ -17441,7 +17437,7 @@
         <v>136</v>
       </c>
       <c r="E389" s="3">
-        <v>40.5</v>
+        <v>40.2</v>
       </c>
       <c r="F389" s="1"/>
       <c r="G389" s="1"/>
@@ -17479,7 +17475,7 @@
         <v>324</v>
       </c>
       <c r="E390" s="3">
-        <v>36.9</v>
+        <v>36.16</v>
       </c>
       <c r="F390" s="1"/>
       <c r="G390" s="1"/>
@@ -17517,7 +17513,7 @@
         <v>325</v>
       </c>
       <c r="E391" s="3">
-        <v>33.3</v>
+        <v>31.8</v>
       </c>
       <c r="F391" s="1"/>
       <c r="G391" s="1"/>
@@ -17593,7 +17589,7 @@
         <v>326</v>
       </c>
       <c r="E393" s="3">
-        <v>27.97</v>
+        <v>27.91</v>
       </c>
       <c r="F393" s="1"/>
       <c r="G393" s="1"/>
@@ -17707,7 +17703,7 @@
         <v>111</v>
       </c>
       <c r="E396" s="3">
-        <v>21.21</v>
+        <v>22.8</v>
       </c>
       <c r="F396" s="1"/>
       <c r="G396" s="1"/>
@@ -17745,7 +17741,7 @@
         <v>118</v>
       </c>
       <c r="E397" s="3">
-        <v>13.9</v>
+        <v>13.8</v>
       </c>
       <c r="F397" s="1"/>
       <c r="G397" s="1"/>
@@ -17897,7 +17893,7 @@
         <v>331</v>
       </c>
       <c r="E401" s="3">
-        <v>19.97</v>
+        <v>19.67</v>
       </c>
       <c r="F401" s="1"/>
       <c r="G401" s="1"/>
@@ -17973,7 +17969,7 @@
         <v>333</v>
       </c>
       <c r="E403" s="3">
-        <v>17.3</v>
+        <v>16.9</v>
       </c>
       <c r="F403" s="1"/>
       <c r="G403" s="1"/>
@@ -18049,7 +18045,7 @@
         <v>179</v>
       </c>
       <c r="E405" s="3">
-        <v>19.3</v>
+        <v>18.8</v>
       </c>
       <c r="F405" s="1"/>
       <c r="G405" s="1"/>
@@ -18087,7 +18083,7 @@
         <v>335</v>
       </c>
       <c r="E406" s="3">
-        <v>18.4</v>
+        <v>18.2</v>
       </c>
       <c r="F406" s="1"/>
       <c r="G406" s="1"/>
@@ -18125,7 +18121,7 @@
         <v>336</v>
       </c>
       <c r="E407" s="3">
-        <v>27.0</v>
+        <v>25.17</v>
       </c>
       <c r="F407" s="1"/>
       <c r="G407" s="1"/>
@@ -18163,7 +18159,7 @@
         <v>337</v>
       </c>
       <c r="E408" s="3">
-        <v>79.41</v>
+        <v>77.61</v>
       </c>
       <c r="F408" s="1"/>
       <c r="G408" s="1"/>
@@ -18201,7 +18197,7 @@
         <v>338</v>
       </c>
       <c r="E409" s="3">
-        <v>36.54</v>
+        <v>35.64</v>
       </c>
       <c r="F409" s="1"/>
       <c r="G409" s="1"/>
@@ -18239,7 +18235,7 @@
         <v>339</v>
       </c>
       <c r="E410" s="3">
-        <v>18.3</v>
+        <v>17.69</v>
       </c>
       <c r="F410" s="1"/>
       <c r="G410" s="1"/>
@@ -18277,7 +18273,7 @@
         <v>340</v>
       </c>
       <c r="E411" s="3">
-        <v>23.17</v>
+        <v>23.07</v>
       </c>
       <c r="F411" s="1"/>
       <c r="G411" s="1"/>
@@ -18315,7 +18311,7 @@
         <v>341</v>
       </c>
       <c r="E412" s="3">
-        <v>23.34</v>
+        <v>22.94</v>
       </c>
       <c r="F412" s="1"/>
       <c r="G412" s="1"/>
@@ -18353,7 +18349,7 @@
         <v>342</v>
       </c>
       <c r="E413" s="3">
-        <v>33.01</v>
+        <v>34.27</v>
       </c>
       <c r="F413" s="1"/>
       <c r="G413" s="1"/>
@@ -18391,7 +18387,7 @@
         <v>343</v>
       </c>
       <c r="E414" s="3">
-        <v>23.3</v>
+        <v>22.5</v>
       </c>
       <c r="F414" s="1"/>
       <c r="G414" s="1"/>
@@ -18429,7 +18425,7 @@
         <v>344</v>
       </c>
       <c r="E415" s="3">
-        <v>35.23</v>
+        <v>34.23</v>
       </c>
       <c r="F415" s="1"/>
       <c r="G415" s="1"/>
@@ -18467,7 +18463,7 @@
         <v>345</v>
       </c>
       <c r="E416" s="3">
-        <v>41.16</v>
+        <v>40.36</v>
       </c>
       <c r="F416" s="1"/>
       <c r="G416" s="1"/>
@@ -18505,7 +18501,7 @@
         <v>346</v>
       </c>
       <c r="E417" s="3">
-        <v>29.67</v>
+        <v>28.47</v>
       </c>
       <c r="F417" s="1"/>
       <c r="G417" s="1"/>
@@ -18543,7 +18539,7 @@
         <v>347</v>
       </c>
       <c r="E418" s="3">
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="F418" s="1"/>
       <c r="G418" s="1"/>
@@ -19911,7 +19907,7 @@
         <v>353</v>
       </c>
       <c r="E454" s="3">
-        <v>34.41</v>
+        <v>33.4</v>
       </c>
       <c r="F454" s="1"/>
       <c r="G454" s="1"/>
@@ -19987,7 +19983,7 @@
         <v>354</v>
       </c>
       <c r="E456" s="3">
-        <v>22.4</v>
+        <v>22.2</v>
       </c>
       <c r="F456" s="1"/>
       <c r="G456" s="1"/>
@@ -20291,7 +20287,7 @@
         <v>362</v>
       </c>
       <c r="E464" s="3">
-        <v>22.5</v>
+        <v>22.0</v>
       </c>
       <c r="F464" s="1"/>
       <c r="G464" s="1"/>
@@ -20671,7 +20667,7 @@
         <v>372</v>
       </c>
       <c r="E474" s="3">
-        <v>38.0</v>
+        <v>37.5</v>
       </c>
       <c r="F474" s="1"/>
       <c r="G474" s="1"/>
@@ -21013,7 +21009,7 @@
         <v>380</v>
       </c>
       <c r="E483" s="3">
-        <v>21.52</v>
+        <v>19.51</v>
       </c>
       <c r="F483" s="1"/>
       <c r="G483" s="1"/>
@@ -21127,7 +21123,7 @@
         <v>383</v>
       </c>
       <c r="E486" s="3">
-        <v>11.25</v>
+        <v>11.0</v>
       </c>
       <c r="F486" s="1"/>
       <c r="G486" s="1"/>
@@ -21165,7 +21161,7 @@
         <v>384</v>
       </c>
       <c r="E487" s="3">
-        <v>40.25</v>
+        <v>40.0</v>
       </c>
       <c r="F487" s="1"/>
       <c r="G487" s="1"/>
@@ -21355,7 +21351,7 @@
         <v>389</v>
       </c>
       <c r="E492" s="3">
-        <v>9.0</v>
+        <v>8.9</v>
       </c>
       <c r="F492" s="1"/>
       <c r="G492" s="1"/>
@@ -21393,7 +21389,7 @@
         <v>390</v>
       </c>
       <c r="E493" s="3">
-        <v>15.52</v>
+        <v>15.34</v>
       </c>
       <c r="F493" s="1"/>
       <c r="G493" s="1"/>
@@ -21431,7 +21427,7 @@
         <v>391</v>
       </c>
       <c r="E494" s="3">
-        <v>9.1</v>
+        <v>9.0</v>
       </c>
       <c r="F494" s="1"/>
       <c r="G494" s="1"/>
@@ -21545,7 +21541,7 @@
         <v>394</v>
       </c>
       <c r="E497" s="3">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="F497" s="1"/>
       <c r="G497" s="1"/>
@@ -21659,7 +21655,7 @@
         <v>397</v>
       </c>
       <c r="E500" s="3">
-        <v>10.4</v>
+        <v>10.3</v>
       </c>
       <c r="F500" s="1"/>
       <c r="G500" s="1"/>
@@ -21811,7 +21807,7 @@
         <v>401</v>
       </c>
       <c r="E504" s="3">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F504" s="1"/>
       <c r="G504" s="1"/>
@@ -21849,7 +21845,7 @@
         <v>402</v>
       </c>
       <c r="E505" s="3">
-        <v>11.0</v>
+        <v>10.9</v>
       </c>
       <c r="F505" s="1"/>
       <c r="G505" s="1"/>
@@ -21887,7 +21883,7 @@
         <v>403</v>
       </c>
       <c r="E506" s="3">
-        <v>11.8</v>
+        <v>11.3</v>
       </c>
       <c r="F506" s="1"/>
       <c r="G506" s="1"/>
@@ -21925,7 +21921,7 @@
         <v>404</v>
       </c>
       <c r="E507" s="3">
-        <v>12.0</v>
+        <v>11.9</v>
       </c>
       <c r="F507" s="1"/>
       <c r="G507" s="1"/>
@@ -22077,7 +22073,7 @@
         <v>408</v>
       </c>
       <c r="E511" s="3">
-        <v>33.0</v>
+        <v>32.2</v>
       </c>
       <c r="F511" s="1"/>
       <c r="G511" s="1"/>
@@ -22761,7 +22757,7 @@
         <v>425</v>
       </c>
       <c r="E529" s="3">
-        <v>10.6</v>
+        <v>10.5</v>
       </c>
       <c r="F529" s="1"/>
       <c r="G529" s="1"/>
@@ -22799,7 +22795,7 @@
         <v>426</v>
       </c>
       <c r="E530" s="3">
-        <v>83.4</v>
+        <v>83.1</v>
       </c>
       <c r="F530" s="1"/>
       <c r="G530" s="1"/>
@@ -22837,7 +22833,7 @@
         <v>427</v>
       </c>
       <c r="E531" s="3">
-        <v>38.62</v>
+        <v>38.35</v>
       </c>
       <c r="F531" s="1"/>
       <c r="G531" s="1"/>
@@ -22913,7 +22909,7 @@
         <v>429</v>
       </c>
       <c r="E533" s="3">
-        <v>20.66</v>
+        <v>20.48</v>
       </c>
       <c r="F533" s="1"/>
       <c r="G533" s="1"/>
@@ -22989,7 +22985,7 @@
         <v>430</v>
       </c>
       <c r="E535" s="3">
-        <v>53.4</v>
+        <v>52.8</v>
       </c>
       <c r="F535" s="1"/>
       <c r="G535" s="1"/>
@@ -23141,7 +23137,7 @@
         <v>434</v>
       </c>
       <c r="E539" s="3">
-        <v>14.9</v>
+        <v>12.6</v>
       </c>
       <c r="F539" s="1"/>
       <c r="G539" s="1"/>
@@ -23179,7 +23175,7 @@
         <v>435</v>
       </c>
       <c r="E540" s="3">
-        <v>16.0</v>
+        <v>13.3</v>
       </c>
       <c r="F540" s="1"/>
       <c r="G540" s="1"/>
@@ -23217,7 +23213,7 @@
         <v>436</v>
       </c>
       <c r="E541" s="3">
-        <v>17.5</v>
+        <v>17.4</v>
       </c>
       <c r="F541" s="1"/>
       <c r="G541" s="1"/>
@@ -23255,7 +23251,7 @@
         <v>437</v>
       </c>
       <c r="E542" s="3">
-        <v>18.4</v>
+        <v>16.1</v>
       </c>
       <c r="F542" s="1"/>
       <c r="G542" s="1"/>
@@ -23293,7 +23289,7 @@
         <v>438</v>
       </c>
       <c r="E543" s="3">
-        <v>10.7</v>
+        <v>10.2</v>
       </c>
       <c r="F543" s="1"/>
       <c r="G543" s="1"/>
@@ -23331,7 +23327,7 @@
         <v>439</v>
       </c>
       <c r="E544" s="3">
-        <v>19.1</v>
+        <v>19.0</v>
       </c>
       <c r="F544" s="1"/>
       <c r="G544" s="1"/>
@@ -23369,7 +23365,7 @@
         <v>440</v>
       </c>
       <c r="E545" s="3">
-        <v>19.5</v>
+        <v>17.15</v>
       </c>
       <c r="F545" s="1"/>
       <c r="G545" s="1"/>
@@ -23483,7 +23479,7 @@
         <v>86</v>
       </c>
       <c r="E548" s="3">
-        <v>13.4</v>
+        <v>13.3</v>
       </c>
       <c r="F548" s="1"/>
       <c r="G548" s="1"/>
@@ -23521,7 +23517,7 @@
         <v>442</v>
       </c>
       <c r="E549" s="3">
-        <v>17.8</v>
+        <v>17.3</v>
       </c>
       <c r="F549" s="1"/>
       <c r="G549" s="1"/>
@@ -23559,7 +23555,7 @@
         <v>443</v>
       </c>
       <c r="E550" s="3">
-        <v>31.6</v>
+        <v>30.0</v>
       </c>
       <c r="F550" s="1"/>
       <c r="G550" s="1"/>
@@ -23711,7 +23707,7 @@
         <v>446</v>
       </c>
       <c r="E554" s="3">
-        <v>16.7</v>
+        <v>16.6</v>
       </c>
       <c r="F554" s="1"/>
       <c r="G554" s="1"/>
@@ -23749,7 +23745,7 @@
         <v>447</v>
       </c>
       <c r="E555" s="3">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
       <c r="F555" s="1"/>
       <c r="G555" s="1"/>
@@ -23977,7 +23973,7 @@
         <v>452</v>
       </c>
       <c r="E561" s="3">
-        <v>16.5</v>
+        <v>16.4</v>
       </c>
       <c r="F561" s="1"/>
       <c r="G561" s="1"/>
@@ -24433,7 +24429,7 @@
         <v>464</v>
       </c>
       <c r="E573" s="3">
-        <v>13.7</v>
+        <v>13.0</v>
       </c>
       <c r="F573" s="1"/>
       <c r="G573" s="1"/>
@@ -24547,7 +24543,7 @@
         <v>466</v>
       </c>
       <c r="E576" s="3">
-        <v>15.4</v>
+        <v>15.3</v>
       </c>
       <c r="F576" s="1"/>
       <c r="G576" s="1"/>
@@ -24775,7 +24771,7 @@
         <v>105</v>
       </c>
       <c r="E582" s="3">
-        <v>21.35</v>
+        <v>20.45</v>
       </c>
       <c r="F582" s="1"/>
       <c r="G582" s="1"/>
@@ -24813,7 +24809,7 @@
         <v>468</v>
       </c>
       <c r="E583" s="3">
-        <v>20.1</v>
+        <v>19.95</v>
       </c>
       <c r="F583" s="1"/>
       <c r="G583" s="1"/>
@@ -24851,7 +24847,7 @@
         <v>469</v>
       </c>
       <c r="E584" s="3">
-        <v>19.9</v>
+        <v>19.8</v>
       </c>
       <c r="F584" s="1"/>
       <c r="G584" s="1"/>
@@ -24965,7 +24961,7 @@
         <v>472</v>
       </c>
       <c r="E587" s="3">
-        <v>18.6</v>
+        <v>18.45</v>
       </c>
       <c r="F587" s="1"/>
       <c r="G587" s="1"/>
@@ -25117,7 +25113,7 @@
         <v>476</v>
       </c>
       <c r="E591" s="3">
-        <v>18.0</v>
+        <v>17.85</v>
       </c>
       <c r="F591" s="1"/>
       <c r="G591" s="1"/>
@@ -25155,7 +25151,7 @@
         <v>477</v>
       </c>
       <c r="E592" s="3">
-        <v>23.1</v>
+        <v>19.19</v>
       </c>
       <c r="F592" s="1"/>
       <c r="G592" s="1"/>
@@ -25231,7 +25227,7 @@
         <v>479</v>
       </c>
       <c r="E594" s="3">
-        <v>24.0</v>
+        <v>23.85</v>
       </c>
       <c r="F594" s="1"/>
       <c r="G594" s="1"/>
@@ -25649,7 +25645,7 @@
         <v>490</v>
       </c>
       <c r="E605" s="3">
-        <v>21.4</v>
+        <v>20.4</v>
       </c>
       <c r="F605" s="1"/>
       <c r="G605" s="1"/>
@@ -25725,7 +25721,7 @@
         <v>492</v>
       </c>
       <c r="E607" s="3">
-        <v>42.0</v>
+        <v>39.6</v>
       </c>
       <c r="F607" s="1"/>
       <c r="G607" s="1"/>
@@ -25877,7 +25873,7 @@
         <v>495</v>
       </c>
       <c r="E611" s="3">
-        <v>29.6</v>
+        <v>28.2</v>
       </c>
       <c r="F611" s="1"/>
       <c r="G611" s="1"/>
@@ -26219,7 +26215,7 @@
         <v>502</v>
       </c>
       <c r="E620" s="3">
-        <v>27.0</v>
+        <v>25.17</v>
       </c>
       <c r="F620" s="1"/>
       <c r="G620" s="1"/>
@@ -26257,7 +26253,7 @@
         <v>502</v>
       </c>
       <c r="E621" s="3">
-        <v>27.0</v>
+        <v>25.17</v>
       </c>
       <c r="F621" s="1"/>
       <c r="G621" s="1"/>
@@ -26295,7 +26291,7 @@
         <v>503</v>
       </c>
       <c r="E622" s="3">
-        <v>78.29</v>
+        <v>75.9</v>
       </c>
       <c r="F622" s="1"/>
       <c r="G622" s="1"/>
@@ -26333,7 +26329,7 @@
         <v>504</v>
       </c>
       <c r="E623" s="3">
-        <v>32.1</v>
+        <v>30.6</v>
       </c>
       <c r="F623" s="1"/>
       <c r="G623" s="1"/>
@@ -26371,7 +26367,7 @@
         <v>505</v>
       </c>
       <c r="E624" s="3">
-        <v>63.0</v>
+        <v>59.4</v>
       </c>
       <c r="F624" s="1"/>
       <c r="G624" s="1"/>
@@ -26485,7 +26481,7 @@
         <v>508</v>
       </c>
       <c r="E627" s="3">
-        <v>38.85</v>
+        <v>37.1</v>
       </c>
       <c r="F627" s="1"/>
       <c r="G627" s="1"/>
@@ -26751,7 +26747,7 @@
         <v>515</v>
       </c>
       <c r="E634" s="3">
-        <v>7.25</v>
+        <v>6.8</v>
       </c>
       <c r="F634" s="1"/>
       <c r="G634" s="1"/>
@@ -26827,7 +26823,7 @@
         <v>517</v>
       </c>
       <c r="E636" s="3">
-        <v>16.2</v>
+        <v>15.4</v>
       </c>
       <c r="F636" s="1"/>
       <c r="G636" s="1"/>
@@ -26865,7 +26861,7 @@
         <v>157</v>
       </c>
       <c r="E637" s="3">
-        <v>10.5</v>
+        <v>9.9</v>
       </c>
       <c r="F637" s="1"/>
       <c r="G637" s="1"/>
@@ -26903,7 +26899,7 @@
         <v>518</v>
       </c>
       <c r="E638" s="3">
-        <v>12.8</v>
+        <v>11.5</v>
       </c>
       <c r="F638" s="1"/>
       <c r="G638" s="1"/>
@@ -26941,7 +26937,7 @@
         <v>519</v>
       </c>
       <c r="E639" s="3">
-        <v>15.8</v>
+        <v>15.0</v>
       </c>
       <c r="F639" s="1"/>
       <c r="G639" s="1"/>
@@ -27017,7 +27013,7 @@
         <v>521</v>
       </c>
       <c r="E641" s="3">
-        <v>8.9</v>
+        <v>8.8</v>
       </c>
       <c r="F641" s="1"/>
       <c r="G641" s="1"/>
@@ -27169,7 +27165,7 @@
         <v>524</v>
       </c>
       <c r="E645" s="3">
-        <v>12.0</v>
+        <v>12.3</v>
       </c>
       <c r="F645" s="1"/>
       <c r="G645" s="1"/>
@@ -27245,7 +27241,7 @@
         <v>525</v>
       </c>
       <c r="E647" s="3">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="F647" s="1"/>
       <c r="G647" s="1"/>
@@ -27511,7 +27507,7 @@
         <v>531</v>
       </c>
       <c r="E654" s="3">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="F654" s="1"/>
       <c r="G654" s="1"/>
@@ -27549,7 +27545,7 @@
         <v>532</v>
       </c>
       <c r="E655" s="3">
-        <v>12.1</v>
+        <v>12.0</v>
       </c>
       <c r="F655" s="1"/>
       <c r="G655" s="1"/>
@@ -27587,7 +27583,7 @@
         <v>533</v>
       </c>
       <c r="E656" s="3">
-        <v>13.0</v>
+        <v>12.9</v>
       </c>
       <c r="F656" s="1"/>
       <c r="G656" s="1"/>
@@ -27701,7 +27697,7 @@
         <v>536</v>
       </c>
       <c r="E659" s="3">
-        <v>11.6</v>
+        <v>11.5</v>
       </c>
       <c r="F659" s="1"/>
       <c r="G659" s="1"/>
@@ -27739,7 +27735,7 @@
         <v>537</v>
       </c>
       <c r="E660" s="3">
-        <v>23.34</v>
+        <v>23.16</v>
       </c>
       <c r="F660" s="1"/>
       <c r="G660" s="1"/>
@@ -27853,7 +27849,7 @@
         <v>540</v>
       </c>
       <c r="E663" s="3">
-        <v>12.0</v>
+        <v>11.6</v>
       </c>
       <c r="F663" s="1"/>
       <c r="G663" s="1"/>
@@ -27891,7 +27887,7 @@
         <v>541</v>
       </c>
       <c r="E664" s="3">
-        <v>16.6</v>
+        <v>16.0</v>
       </c>
       <c r="F664" s="1"/>
       <c r="G664" s="1"/>
@@ -28081,7 +28077,7 @@
         <v>546</v>
       </c>
       <c r="E669" s="3">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="F669" s="1"/>
       <c r="G669" s="1"/>
@@ -28347,7 +28343,7 @@
         <v>551</v>
       </c>
       <c r="E676" s="3">
-        <v>14.5</v>
+        <v>14.4</v>
       </c>
       <c r="F676" s="1"/>
       <c r="G676" s="1"/>
@@ -28613,7 +28609,7 @@
         <v>555</v>
       </c>
       <c r="E683" s="3">
-        <v>18.4</v>
+        <v>16.1</v>
       </c>
       <c r="F683" s="1"/>
       <c r="G683" s="1"/>
@@ -28651,7 +28647,7 @@
         <v>556</v>
       </c>
       <c r="E684" s="3">
-        <v>16.42</v>
+        <v>16.12</v>
       </c>
       <c r="F684" s="1"/>
       <c r="G684" s="1"/>
@@ -28689,7 +28685,7 @@
         <v>557</v>
       </c>
       <c r="E685" s="3">
-        <v>29.74</v>
+        <v>29.34</v>
       </c>
       <c r="F685" s="1"/>
       <c r="G685" s="1"/>
@@ -28727,7 +28723,7 @@
         <v>558</v>
       </c>
       <c r="E686" s="3">
-        <v>29.0</v>
+        <v>26.49</v>
       </c>
       <c r="F686" s="1"/>
       <c r="G686" s="1"/>
@@ -28765,7 +28761,7 @@
         <v>560</v>
       </c>
       <c r="E687" s="3">
-        <v>19.7</v>
+        <v>17.5</v>
       </c>
       <c r="F687" s="1"/>
       <c r="G687" s="1"/>
@@ -28803,7 +28799,7 @@
         <v>561</v>
       </c>
       <c r="E688" s="3">
-        <v>29.55</v>
+        <v>26.25</v>
       </c>
       <c r="F688" s="1"/>
       <c r="G688" s="1"/>
@@ -28841,7 +28837,7 @@
         <v>559</v>
       </c>
       <c r="E689" s="3">
-        <v>39.4</v>
+        <v>35.0</v>
       </c>
       <c r="F689" s="1"/>
       <c r="G689" s="1"/>
@@ -28879,7 +28875,7 @@
         <v>562</v>
       </c>
       <c r="E690" s="3">
-        <v>59.1</v>
+        <v>52.5</v>
       </c>
       <c r="F690" s="1"/>
       <c r="G690" s="1"/>
@@ -29221,7 +29217,7 @@
         <v>176</v>
       </c>
       <c r="E699" s="3">
-        <v>14.9</v>
+        <v>14.8</v>
       </c>
       <c r="F699" s="1"/>
       <c r="G699" s="1"/>
@@ -29259,7 +29255,7 @@
         <v>572</v>
       </c>
       <c r="E700" s="3">
-        <v>7.22</v>
+        <v>7.13</v>
       </c>
       <c r="F700" s="1"/>
       <c r="G700" s="1"/>
@@ -29297,7 +29293,7 @@
         <v>573</v>
       </c>
       <c r="E701" s="3">
-        <v>7.7</v>
+        <v>7.63</v>
       </c>
       <c r="F701" s="1"/>
       <c r="G701" s="1"/>
@@ -29373,7 +29369,7 @@
         <v>575</v>
       </c>
       <c r="E703" s="3">
-        <v>42.0</v>
+        <v>41.7</v>
       </c>
       <c r="F703" s="1"/>
       <c r="G703" s="1"/>
@@ -29411,7 +29407,7 @@
         <v>576</v>
       </c>
       <c r="E704" s="3">
-        <v>104.6</v>
+        <v>104.4</v>
       </c>
       <c r="F704" s="1"/>
       <c r="G704" s="1"/>
@@ -29449,7 +29445,7 @@
         <v>577</v>
       </c>
       <c r="E705" s="3">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F705" s="1"/>
       <c r="G705" s="1"/>
@@ -29487,7 +29483,7 @@
         <v>578</v>
       </c>
       <c r="E706" s="3">
-        <v>13.2</v>
+        <v>13.1</v>
       </c>
       <c r="F706" s="1"/>
       <c r="G706" s="1"/>
@@ -29601,7 +29597,7 @@
         <v>580</v>
       </c>
       <c r="E709" s="3">
-        <v>23.6</v>
+        <v>23.4</v>
       </c>
       <c r="F709" s="1"/>
       <c r="G709" s="1"/>
@@ -29677,7 +29673,7 @@
         <v>582</v>
       </c>
       <c r="E711" s="3">
-        <v>29.0</v>
+        <v>26.5</v>
       </c>
       <c r="F711" s="1"/>
       <c r="G711" s="1"/>
@@ -29714,9 +29710,7 @@
       <c r="D712" s="4" t="s">
         <v>583</v>
       </c>
-      <c r="E712" s="3">
-        <v>10.82</v>
-      </c>
+      <c r="E712" s="3"/>
       <c r="F712" s="1"/>
       <c r="G712" s="1"/>
       <c r="H712" s="1"/>
@@ -29829,7 +29823,7 @@
         <v>179</v>
       </c>
       <c r="E715" s="3">
-        <v>19.3</v>
+        <v>18.8</v>
       </c>
       <c r="F715" s="1"/>
       <c r="G715" s="1"/>
@@ -29867,7 +29861,7 @@
         <v>586</v>
       </c>
       <c r="E716" s="3">
-        <v>15.8</v>
+        <v>15.2</v>
       </c>
       <c r="F716" s="1"/>
       <c r="G716" s="1"/>
@@ -29905,7 +29899,7 @@
         <v>587</v>
       </c>
       <c r="E717" s="3">
-        <v>16.1</v>
+        <v>14.0</v>
       </c>
       <c r="F717" s="1"/>
       <c r="G717" s="1"/>
@@ -29943,7 +29937,7 @@
         <v>588</v>
       </c>
       <c r="E718" s="3">
-        <v>27.52</v>
+        <v>26.77</v>
       </c>
       <c r="F718" s="1"/>
       <c r="G718" s="1"/>
@@ -29981,7 +29975,7 @@
         <v>589</v>
       </c>
       <c r="E719" s="3">
-        <v>26.7</v>
+        <v>26.17</v>
       </c>
       <c r="F719" s="1"/>
       <c r="G719" s="1"/>
@@ -30019,7 +30013,7 @@
         <v>590</v>
       </c>
       <c r="E720" s="3">
-        <v>17.0</v>
+        <v>15.4</v>
       </c>
       <c r="F720" s="1"/>
       <c r="G720" s="1"/>
@@ -30057,7 +30051,7 @@
         <v>180</v>
       </c>
       <c r="E721" s="3">
-        <v>36.8</v>
+        <v>31.82</v>
       </c>
       <c r="F721" s="1"/>
       <c r="G721" s="1"/>
@@ -30095,7 +30089,7 @@
         <v>591</v>
       </c>
       <c r="E722" s="3">
-        <v>40.54</v>
+        <v>39.54</v>
       </c>
       <c r="F722" s="1"/>
       <c r="G722" s="1"/>
@@ -30133,7 +30127,7 @@
         <v>592</v>
       </c>
       <c r="E723" s="3">
-        <v>34.8</v>
+        <v>34.1</v>
       </c>
       <c r="F723" s="1"/>
       <c r="G723" s="1"/>
@@ -30171,7 +30165,7 @@
         <v>593</v>
       </c>
       <c r="E724" s="3">
-        <v>21.25</v>
+        <v>19.25</v>
       </c>
       <c r="F724" s="1"/>
       <c r="G724" s="1"/>
@@ -30209,7 +30203,7 @@
         <v>594</v>
       </c>
       <c r="E725" s="3">
-        <v>47.0</v>
+        <v>46.5</v>
       </c>
       <c r="F725" s="1"/>
       <c r="G725" s="1"/>
@@ -30247,7 +30241,7 @@
         <v>595</v>
       </c>
       <c r="E726" s="3">
-        <v>57.6</v>
+        <v>56.7</v>
       </c>
       <c r="F726" s="1"/>
       <c r="G726" s="1"/>
@@ -30285,7 +30279,7 @@
         <v>596</v>
       </c>
       <c r="E727" s="3">
-        <v>48.0</v>
+        <v>44.45</v>
       </c>
       <c r="F727" s="1"/>
       <c r="G727" s="1"/>
@@ -30323,7 +30317,7 @@
         <v>597</v>
       </c>
       <c r="E728" s="3">
-        <v>12.0</v>
+        <v>11.49</v>
       </c>
       <c r="F728" s="1"/>
       <c r="G728" s="1"/>
@@ -30361,7 +30355,7 @@
         <v>598</v>
       </c>
       <c r="E729" s="3">
-        <v>16.1</v>
+        <v>15.39</v>
       </c>
       <c r="F729" s="1"/>
       <c r="G729" s="1"/>
@@ -30399,7 +30393,7 @@
         <v>599</v>
       </c>
       <c r="E730" s="3">
-        <v>18.6</v>
+        <v>16.04</v>
       </c>
       <c r="F730" s="1"/>
       <c r="G730" s="1"/>
@@ -30437,7 +30431,7 @@
         <v>600</v>
       </c>
       <c r="E731" s="3">
-        <v>55.8</v>
+        <v>48.11</v>
       </c>
       <c r="F731" s="1"/>
       <c r="G731" s="1"/>
@@ -30475,7 +30469,7 @@
         <v>601</v>
       </c>
       <c r="E732" s="3">
-        <v>27.9</v>
+        <v>24.06</v>
       </c>
       <c r="F732" s="1"/>
       <c r="G732" s="1"/>
@@ -30513,7 +30507,7 @@
         <v>602</v>
       </c>
       <c r="E733" s="3">
-        <v>37.2</v>
+        <v>32.07</v>
       </c>
       <c r="F733" s="1"/>
       <c r="G733" s="1"/>
@@ -30551,7 +30545,7 @@
         <v>604</v>
       </c>
       <c r="E734" s="3">
-        <v>18.6</v>
+        <v>16.04</v>
       </c>
       <c r="F734" s="1"/>
       <c r="G734" s="1"/>
@@ -30589,7 +30583,7 @@
         <v>603</v>
       </c>
       <c r="E735" s="3">
-        <v>27.9</v>
+        <v>24.06</v>
       </c>
       <c r="F735" s="1"/>
       <c r="G735" s="1"/>
@@ -30627,7 +30621,7 @@
         <v>605</v>
       </c>
       <c r="E736" s="3">
-        <v>37.2</v>
+        <v>32.07</v>
       </c>
       <c r="F736" s="1"/>
       <c r="G736" s="1"/>
@@ -30665,7 +30659,7 @@
         <v>606</v>
       </c>
       <c r="E737" s="3">
-        <v>55.8</v>
+        <v>48.11</v>
       </c>
       <c r="F737" s="1"/>
       <c r="G737" s="1"/>
@@ -30703,7 +30697,7 @@
         <v>607</v>
       </c>
       <c r="E738" s="3">
-        <v>40.5</v>
+        <v>39.0</v>
       </c>
       <c r="F738" s="1"/>
       <c r="G738" s="1"/>
@@ -30741,7 +30735,7 @@
         <v>608</v>
       </c>
       <c r="E739" s="3">
-        <v>25.5</v>
+        <v>25.1</v>
       </c>
       <c r="F739" s="1"/>
       <c r="G739" s="1"/>
@@ -30779,7 +30773,7 @@
         <v>609</v>
       </c>
       <c r="E740" s="3">
-        <v>40.6</v>
+        <v>39.57</v>
       </c>
       <c r="F740" s="1"/>
       <c r="G740" s="1"/>
@@ -30817,7 +30811,7 @@
         <v>611</v>
       </c>
       <c r="E741" s="3">
-        <v>17.7</v>
+        <v>14.95</v>
       </c>
       <c r="F741" s="1"/>
       <c r="G741" s="1"/>
@@ -30855,7 +30849,7 @@
         <v>612</v>
       </c>
       <c r="E742" s="3">
-        <v>26.55</v>
+        <v>22.42</v>
       </c>
       <c r="F742" s="1"/>
       <c r="G742" s="1"/>
@@ -30893,7 +30887,7 @@
         <v>610</v>
       </c>
       <c r="E743" s="3">
-        <v>35.4</v>
+        <v>29.9</v>
       </c>
       <c r="F743" s="1"/>
       <c r="G743" s="1"/>
@@ -30931,7 +30925,7 @@
         <v>613</v>
       </c>
       <c r="E744" s="3">
-        <v>53.1</v>
+        <v>44.85</v>
       </c>
       <c r="F744" s="1"/>
       <c r="G744" s="1"/>
@@ -30969,7 +30963,7 @@
         <v>615</v>
       </c>
       <c r="E745" s="3">
-        <v>19.5</v>
+        <v>17.2</v>
       </c>
       <c r="F745" s="1"/>
       <c r="G745" s="1"/>
@@ -31007,7 +31001,7 @@
         <v>614</v>
       </c>
       <c r="E746" s="3">
-        <v>39.0</v>
+        <v>34.4</v>
       </c>
       <c r="F746" s="1"/>
       <c r="G746" s="1"/>
@@ -31045,7 +31039,7 @@
         <v>616</v>
       </c>
       <c r="E747" s="3">
-        <v>58.5</v>
+        <v>51.6</v>
       </c>
       <c r="F747" s="1"/>
       <c r="G747" s="1"/>
@@ -31083,7 +31077,7 @@
         <v>617</v>
       </c>
       <c r="E748" s="3">
-        <v>34.0</v>
+        <v>32.29</v>
       </c>
       <c r="F748" s="1"/>
       <c r="G748" s="1"/>
@@ -31121,7 +31115,7 @@
         <v>618</v>
       </c>
       <c r="E749" s="3">
-        <v>19.74</v>
+        <v>18.69</v>
       </c>
       <c r="F749" s="1"/>
       <c r="G749" s="1"/>
@@ -31159,7 +31153,7 @@
         <v>619</v>
       </c>
       <c r="E750" s="3">
-        <v>20.2</v>
+        <v>17.86</v>
       </c>
       <c r="F750" s="1"/>
       <c r="G750" s="1"/>
@@ -31197,7 +31191,7 @@
         <v>620</v>
       </c>
       <c r="E751" s="3">
-        <v>30.3</v>
+        <v>26.79</v>
       </c>
       <c r="F751" s="1"/>
       <c r="G751" s="1"/>
@@ -31235,7 +31229,7 @@
         <v>621</v>
       </c>
       <c r="E752" s="3">
-        <v>40.4</v>
+        <v>35.72</v>
       </c>
       <c r="F752" s="1"/>
       <c r="G752" s="1"/>
@@ -31273,7 +31267,7 @@
         <v>622</v>
       </c>
       <c r="E753" s="3">
-        <v>60.6</v>
+        <v>53.58</v>
       </c>
       <c r="F753" s="1"/>
       <c r="G753" s="1"/>
@@ -31311,7 +31305,7 @@
         <v>623</v>
       </c>
       <c r="E754" s="3">
-        <v>37.8</v>
+        <v>33.52</v>
       </c>
       <c r="F754" s="1"/>
       <c r="G754" s="1"/>
@@ -31349,7 +31343,7 @@
         <v>624</v>
       </c>
       <c r="E755" s="3">
-        <v>26.4</v>
+        <v>26.2</v>
       </c>
       <c r="F755" s="1"/>
       <c r="G755" s="1"/>
@@ -31387,7 +31381,7 @@
         <v>625</v>
       </c>
       <c r="E756" s="3">
-        <v>31.5</v>
+        <v>30.42</v>
       </c>
       <c r="F756" s="1"/>
       <c r="G756" s="1"/>
@@ -31425,7 +31419,7 @@
         <v>188</v>
       </c>
       <c r="E757" s="3">
-        <v>11.9</v>
+        <v>11.8</v>
       </c>
       <c r="F757" s="1"/>
       <c r="G757" s="1"/>
@@ -31653,7 +31647,7 @@
         <v>630</v>
       </c>
       <c r="E763" s="3">
-        <v>8.2</v>
+        <v>8.1</v>
       </c>
       <c r="F763" s="1"/>
       <c r="G763" s="1"/>
@@ -31729,7 +31723,7 @@
         <v>632</v>
       </c>
       <c r="E765" s="3">
-        <v>39.0</v>
+        <v>37.29</v>
       </c>
       <c r="F765" s="1"/>
       <c r="G765" s="1"/>
@@ -31767,7 +31761,7 @@
         <v>633</v>
       </c>
       <c r="E766" s="3">
-        <v>43.4</v>
+        <v>41.39</v>
       </c>
       <c r="F766" s="1"/>
       <c r="G766" s="1"/>
@@ -31805,7 +31799,7 @@
         <v>634</v>
       </c>
       <c r="E767" s="3">
-        <v>12.4</v>
+        <v>12.3</v>
       </c>
       <c r="F767" s="1"/>
       <c r="G767" s="1"/>
@@ -31919,7 +31913,7 @@
         <v>637</v>
       </c>
       <c r="E770" s="3">
-        <v>18.2</v>
+        <v>18.0</v>
       </c>
       <c r="F770" s="1"/>
       <c r="G770" s="1"/>
@@ -32337,7 +32331,7 @@
         <v>648</v>
       </c>
       <c r="E781" s="3">
-        <v>29.0</v>
+        <v>27.2</v>
       </c>
       <c r="F781" s="1"/>
       <c r="G781" s="1"/>
@@ -32375,7 +32369,7 @@
         <v>649</v>
       </c>
       <c r="E782" s="3">
-        <v>14.5</v>
+        <v>13.6</v>
       </c>
       <c r="F782" s="1"/>
       <c r="G782" s="1"/>
@@ -32527,7 +32521,7 @@
         <v>652</v>
       </c>
       <c r="E786" s="3">
-        <v>22.0</v>
+        <v>19.6</v>
       </c>
       <c r="F786" s="1"/>
       <c r="G786" s="1"/>
@@ -32565,7 +32559,7 @@
         <v>653</v>
       </c>
       <c r="E787" s="3">
-        <v>44.0</v>
+        <v>39.19</v>
       </c>
       <c r="F787" s="1"/>
       <c r="G787" s="1"/>
@@ -32603,7 +32597,7 @@
         <v>654</v>
       </c>
       <c r="E788" s="3">
-        <v>33.0</v>
+        <v>29.39</v>
       </c>
       <c r="F788" s="1"/>
       <c r="G788" s="1"/>
@@ -32641,7 +32635,7 @@
         <v>655</v>
       </c>
       <c r="E789" s="3">
-        <v>66.0</v>
+        <v>58.79</v>
       </c>
       <c r="F789" s="1"/>
       <c r="G789" s="1"/>
@@ -32679,7 +32673,7 @@
         <v>656</v>
       </c>
       <c r="E790" s="3">
-        <v>8.2</v>
+        <v>8.1</v>
       </c>
       <c r="F790" s="1"/>
       <c r="G790" s="1"/>
@@ -32755,7 +32749,7 @@
         <v>658</v>
       </c>
       <c r="E792" s="3">
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="F792" s="1"/>
       <c r="G792" s="1"/>
@@ -33059,7 +33053,7 @@
         <v>666</v>
       </c>
       <c r="E800" s="3">
-        <v>11.2</v>
+        <v>10.89</v>
       </c>
       <c r="F800" s="1"/>
       <c r="G800" s="1"/>
@@ -33173,7 +33167,7 @@
         <v>669</v>
       </c>
       <c r="E803" s="3">
-        <v>35.0</v>
+        <v>32.69</v>
       </c>
       <c r="F803" s="1"/>
       <c r="G803" s="1"/>
@@ -33211,7 +33205,7 @@
         <v>670</v>
       </c>
       <c r="E804" s="3">
-        <v>12.4</v>
+        <v>11.89</v>
       </c>
       <c r="F804" s="1"/>
       <c r="G804" s="1"/>
@@ -33591,7 +33585,7 @@
         <v>679</v>
       </c>
       <c r="E814" s="3">
-        <v>29.7</v>
+        <v>29.5</v>
       </c>
       <c r="F814" s="1"/>
       <c r="G814" s="1"/>
@@ -33667,7 +33661,7 @@
         <v>681</v>
       </c>
       <c r="E816" s="3">
-        <v>39.6</v>
+        <v>37.4</v>
       </c>
       <c r="F816" s="1"/>
       <c r="G816" s="1"/>
@@ -33781,7 +33775,7 @@
         <v>684</v>
       </c>
       <c r="E819" s="3">
-        <v>21.0</v>
+        <v>20.75</v>
       </c>
       <c r="F819" s="1"/>
       <c r="G819" s="1"/>
@@ -33857,7 +33851,7 @@
         <v>686</v>
       </c>
       <c r="E821" s="3">
-        <v>16.2</v>
+        <v>16.1</v>
       </c>
       <c r="F821" s="1"/>
       <c r="G821" s="1"/>
@@ -34237,7 +34231,7 @@
         <v>695</v>
       </c>
       <c r="E831" s="3">
-        <v>270.0</v>
+        <v>264.0</v>
       </c>
       <c r="F831" s="1"/>
       <c r="G831" s="1"/>
@@ -34275,7 +34269,7 @@
         <v>696</v>
       </c>
       <c r="E832" s="3">
-        <v>13.0</v>
+        <v>12.9</v>
       </c>
       <c r="F832" s="1"/>
       <c r="G832" s="1"/>
@@ -34389,7 +34383,7 @@
         <v>699</v>
       </c>
       <c r="E835" s="3">
-        <v>22.2</v>
+        <v>19.95</v>
       </c>
       <c r="F835" s="1"/>
       <c r="G835" s="1"/>
@@ -34427,7 +34421,7 @@
         <v>700</v>
       </c>
       <c r="E836" s="3">
-        <v>25.95</v>
+        <v>22.42</v>
       </c>
       <c r="F836" s="1"/>
       <c r="G836" s="1"/>
@@ -34465,7 +34459,7 @@
         <v>701</v>
       </c>
       <c r="E837" s="3">
-        <v>51.9</v>
+        <v>44.85</v>
       </c>
       <c r="F837" s="1"/>
       <c r="G837" s="1"/>
@@ -34503,7 +34497,7 @@
         <v>702</v>
       </c>
       <c r="E838" s="3">
-        <v>17.3</v>
+        <v>14.95</v>
       </c>
       <c r="F838" s="1"/>
       <c r="G838" s="1"/>
@@ -34541,7 +34535,7 @@
         <v>703</v>
       </c>
       <c r="E839" s="3">
-        <v>34.6</v>
+        <v>29.9</v>
       </c>
       <c r="F839" s="1"/>
       <c r="G839" s="1"/>
@@ -34579,7 +34573,7 @@
         <v>704</v>
       </c>
       <c r="E840" s="3">
-        <v>22.4</v>
+        <v>19.8</v>
       </c>
       <c r="F840" s="1"/>
       <c r="G840" s="1"/>
@@ -34617,7 +34611,7 @@
         <v>705</v>
       </c>
       <c r="E841" s="3">
-        <v>25.65</v>
+        <v>25.5</v>
       </c>
       <c r="F841" s="1"/>
       <c r="G841" s="1"/>
@@ -34692,9 +34686,7 @@
       <c r="D843" s="4" t="s">
         <v>707</v>
       </c>
-      <c r="E843" s="3">
-        <v>7.98</v>
-      </c>
+      <c r="E843" s="3"/>
       <c r="F843" s="1"/>
       <c r="G843" s="1"/>
       <c r="H843" s="1"/>
@@ -34845,7 +34837,7 @@
         <v>711</v>
       </c>
       <c r="E847" s="3">
-        <v>10.9</v>
+        <v>10.8</v>
       </c>
       <c r="F847" s="1"/>
       <c r="G847" s="1"/>
@@ -34883,7 +34875,7 @@
         <v>712</v>
       </c>
       <c r="E848" s="3">
-        <v>9.0</v>
+        <v>8.9</v>
       </c>
       <c r="F848" s="1"/>
       <c r="G848" s="1"/>
@@ -34921,7 +34913,7 @@
         <v>713</v>
       </c>
       <c r="E849" s="3">
-        <v>25.6</v>
+        <v>25.4</v>
       </c>
       <c r="F849" s="1"/>
       <c r="G849" s="1"/>
@@ -35035,7 +35027,7 @@
         <v>716</v>
       </c>
       <c r="E852" s="3">
-        <v>7.74</v>
+        <v>7.68</v>
       </c>
       <c r="F852" s="1"/>
       <c r="G852" s="1"/>
@@ -35339,7 +35331,7 @@
         <v>723</v>
       </c>
       <c r="E860" s="3">
-        <v>35.02</v>
+        <v>32.04</v>
       </c>
       <c r="F860" s="1"/>
       <c r="G860" s="1"/>
@@ -35491,7 +35483,7 @@
         <v>347</v>
       </c>
       <c r="E864" s="3">
-        <v>9.4</v>
+        <v>9.3</v>
       </c>
       <c r="F864" s="1"/>
       <c r="G864" s="1"/>
@@ -35529,7 +35521,7 @@
         <v>727</v>
       </c>
       <c r="E865" s="3">
-        <v>9.0</v>
+        <v>8.8</v>
       </c>
       <c r="F865" s="1"/>
       <c r="G865" s="1"/>
@@ -35567,7 +35559,7 @@
         <v>727</v>
       </c>
       <c r="E866" s="3">
-        <v>9.0</v>
+        <v>8.8</v>
       </c>
       <c r="F866" s="1"/>
       <c r="G866" s="1"/>
@@ -35757,7 +35749,7 @@
         <v>732</v>
       </c>
       <c r="E871" s="3">
-        <v>18.6</v>
+        <v>18.45</v>
       </c>
       <c r="F871" s="1"/>
       <c r="G871" s="1"/>
@@ -35833,7 +35825,7 @@
         <v>734</v>
       </c>
       <c r="E873" s="3">
-        <v>8.55</v>
+        <v>8.5</v>
       </c>
       <c r="F873" s="1"/>
       <c r="G873" s="1"/>
@@ -35871,7 +35863,7 @@
         <v>735</v>
       </c>
       <c r="E874" s="3">
-        <v>16.55</v>
+        <v>16.45</v>
       </c>
       <c r="F874" s="1"/>
       <c r="G874" s="1"/>
@@ -35947,7 +35939,7 @@
         <v>737</v>
       </c>
       <c r="E876" s="3">
-        <v>11.2</v>
+        <v>11.1</v>
       </c>
       <c r="F876" s="1"/>
       <c r="G876" s="1"/>
@@ -35985,7 +35977,7 @@
         <v>738</v>
       </c>
       <c r="E877" s="3">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="F877" s="1"/>
       <c r="G877" s="1"/>
@@ -36061,7 +36053,7 @@
         <v>740</v>
       </c>
       <c r="E879" s="3">
-        <v>13.1</v>
+        <v>13.0</v>
       </c>
       <c r="F879" s="1"/>
       <c r="G879" s="1"/>
@@ -36099,7 +36091,7 @@
         <v>741</v>
       </c>
       <c r="E880" s="3">
-        <v>16.4</v>
+        <v>16.3</v>
       </c>
       <c r="F880" s="1"/>
       <c r="G880" s="1"/>
@@ -36365,7 +36357,7 @@
         <v>748</v>
       </c>
       <c r="E887" s="3">
-        <v>12.3</v>
+        <v>12.15</v>
       </c>
       <c r="F887" s="1"/>
       <c r="G887" s="1"/>
@@ -36441,7 +36433,7 @@
         <v>750</v>
       </c>
       <c r="E889" s="3">
-        <v>98.71</v>
+        <v>98.4</v>
       </c>
       <c r="F889" s="1"/>
       <c r="G889" s="1"/>
@@ -36631,7 +36623,7 @@
         <v>754</v>
       </c>
       <c r="E894" s="3">
-        <v>10.7</v>
+        <v>10.6</v>
       </c>
       <c r="F894" s="1"/>
       <c r="G894" s="1"/>
@@ -36707,7 +36699,7 @@
         <v>756</v>
       </c>
       <c r="E896" s="3">
-        <v>8.8</v>
+        <v>8.7</v>
       </c>
       <c r="F896" s="1"/>
       <c r="G896" s="1"/>
@@ -36783,7 +36775,7 @@
         <v>758</v>
       </c>
       <c r="E898" s="3">
-        <v>23.0</v>
+        <v>22.8</v>
       </c>
       <c r="F898" s="1"/>
       <c r="G898" s="1"/>
@@ -36859,7 +36851,7 @@
         <v>760</v>
       </c>
       <c r="E900" s="3">
-        <v>155.5</v>
+        <v>148.0</v>
       </c>
       <c r="F900" s="1"/>
       <c r="G900" s="1"/>
@@ -37011,7 +37003,7 @@
         <v>764</v>
       </c>
       <c r="E904" s="3">
-        <v>30.8</v>
+        <v>30.7</v>
       </c>
       <c r="F904" s="1"/>
       <c r="G904" s="1"/>
@@ -37049,7 +37041,7 @@
         <v>765</v>
       </c>
       <c r="E905" s="3">
-        <v>52.0</v>
+        <v>51.5</v>
       </c>
       <c r="F905" s="1"/>
       <c r="G905" s="1"/>
@@ -37087,7 +37079,7 @@
         <v>766</v>
       </c>
       <c r="E906" s="3">
-        <v>17.1</v>
+        <v>17.0</v>
       </c>
       <c r="F906" s="1"/>
       <c r="G906" s="1"/>
@@ -37163,7 +37155,7 @@
         <v>768</v>
       </c>
       <c r="E908" s="3">
-        <v>14.4</v>
+        <v>14.2</v>
       </c>
       <c r="F908" s="1"/>
       <c r="G908" s="1"/>
@@ -37277,7 +37269,7 @@
         <v>771</v>
       </c>
       <c r="E911" s="3">
-        <v>14.9</v>
+        <v>15.0</v>
       </c>
       <c r="F911" s="1"/>
       <c r="G911" s="1"/>
@@ -37315,7 +37307,7 @@
         <v>772</v>
       </c>
       <c r="E912" s="3">
-        <v>17.6</v>
+        <v>17.5</v>
       </c>
       <c r="F912" s="1"/>
       <c r="G912" s="1"/>
@@ -37543,7 +37535,7 @@
         <v>778</v>
       </c>
       <c r="E918" s="3">
-        <v>21.5</v>
+        <v>21.4</v>
       </c>
       <c r="F918" s="1"/>
       <c r="G918" s="1"/>
@@ -37657,7 +37649,7 @@
         <v>781</v>
       </c>
       <c r="E921" s="3">
-        <v>13.1</v>
+        <v>12.8</v>
       </c>
       <c r="F921" s="1"/>
       <c r="G921" s="1"/>
@@ -37695,7 +37687,7 @@
         <v>782</v>
       </c>
       <c r="E922" s="3">
-        <v>4.5</v>
+        <v>4.45</v>
       </c>
       <c r="F922" s="1"/>
       <c r="G922" s="1"/>
@@ -37847,7 +37839,7 @@
         <v>785</v>
       </c>
       <c r="E926" s="3">
-        <v>15.8</v>
+        <v>15.7</v>
       </c>
       <c r="F926" s="1"/>
       <c r="G926" s="1"/>
@@ -37885,7 +37877,7 @@
         <v>786</v>
       </c>
       <c r="E927" s="3">
-        <v>23.1</v>
+        <v>22.9</v>
       </c>
       <c r="F927" s="1"/>
       <c r="G927" s="1"/>
@@ -37961,7 +37953,7 @@
         <v>788</v>
       </c>
       <c r="E929" s="3">
-        <v>12.8</v>
+        <v>12.7</v>
       </c>
       <c r="F929" s="1"/>
       <c r="G929" s="1"/>
@@ -38075,7 +38067,7 @@
         <v>791</v>
       </c>
       <c r="E932" s="3">
-        <v>15.9</v>
+        <v>15.8</v>
       </c>
       <c r="F932" s="1"/>
       <c r="G932" s="1"/>
@@ -38303,7 +38295,7 @@
         <v>797</v>
       </c>
       <c r="E938" s="3">
-        <v>8.3</v>
+        <v>8.2</v>
       </c>
       <c r="F938" s="1"/>
       <c r="G938" s="1"/>
@@ -38455,7 +38447,7 @@
         <v>801</v>
       </c>
       <c r="E942" s="3">
-        <v>28.7</v>
+        <v>28.6</v>
       </c>
       <c r="F942" s="1"/>
       <c r="G942" s="1"/>
@@ -38493,7 +38485,7 @@
         <v>802</v>
       </c>
       <c r="E943" s="3">
-        <v>18.2</v>
+        <v>18.1</v>
       </c>
       <c r="F943" s="1"/>
       <c r="G943" s="1"/>

</xml_diff>